<commit_message>
# add more stocks
</commit_message>
<xml_diff>
--- a/data/stocks_20260206_095242.xlsx
+++ b/data/stocks_20260206_095242.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="股票池" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:T39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,10 +519,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>000858</t>
-        </is>
+      <c r="A2" t="n">
+        <v>858</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -587,10 +585,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>300750</t>
-        </is>
+      <c r="A3" t="n">
+        <v>300750</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -655,10 +651,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>600030</t>
-        </is>
+      <c r="A4" t="n">
+        <v>600030</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -723,10 +717,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>600118</t>
-        </is>
+      <c r="A5" t="n">
+        <v>600118</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -791,10 +783,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>300308</t>
-        </is>
+      <c r="A6" t="n">
+        <v>300308</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -859,10 +849,8 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>601398</t>
-        </is>
+      <c r="A7" t="n">
+        <v>601398</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -927,10 +915,8 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>601919</t>
-        </is>
+      <c r="A8" t="n">
+        <v>601919</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -995,10 +981,8 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>002261</t>
-        </is>
+      <c r="A9" t="n">
+        <v>2261</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,10 +1047,8 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>688041</t>
-        </is>
+      <c r="A10" t="n">
+        <v>688041</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1131,10 +1113,8 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>300502</t>
-        </is>
+      <c r="A11" t="n">
+        <v>300502</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1199,10 +1179,8 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>300394</t>
-        </is>
+      <c r="A12" t="n">
+        <v>300394</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1267,10 +1245,8 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>000988</t>
-        </is>
+      <c r="A13" t="n">
+        <v>988</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1335,10 +1311,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>603986</t>
-        </is>
+      <c r="A14" t="n">
+        <v>603986</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1403,10 +1377,8 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>688525</t>
-        </is>
+      <c r="A15" t="n">
+        <v>688525</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1471,10 +1443,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>300042</t>
-        </is>
+      <c r="A16" t="n">
+        <v>300042</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1539,10 +1509,8 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>300302</t>
-        </is>
+      <c r="A17" t="n">
+        <v>300302</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1607,10 +1575,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>000020</t>
-        </is>
+      <c r="A18" t="n">
+        <v>20</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1675,10 +1641,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>603881</t>
-        </is>
+      <c r="A19" t="n">
+        <v>603881</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1743,10 +1707,8 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>300017</t>
-        </is>
+      <c r="A20" t="n">
+        <v>300017</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1811,10 +1773,8 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>300418</t>
-        </is>
+      <c r="A21" t="n">
+        <v>300418</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1879,10 +1839,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>002230</t>
-        </is>
+      <c r="A22" t="n">
+        <v>2230</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1947,10 +1905,8 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>300058</t>
-        </is>
+      <c r="A23" t="n">
+        <v>300058</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2015,10 +1971,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>300496</t>
-        </is>
+      <c r="A24" t="n">
+        <v>300496</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2083,10 +2037,8 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>000547</t>
-        </is>
+      <c r="A25" t="n">
+        <v>547</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2151,10 +2103,8 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>002202</t>
-        </is>
+      <c r="A26" t="n">
+        <v>2202</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2219,10 +2169,8 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>301128</t>
-        </is>
+      <c r="A27" t="n">
+        <v>301128</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2281,6 +2229,774 @@
         <v>3.46</v>
       </c>
       <c r="T27" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>601899</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>紫金矿业</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>37.19</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="E28" t="n">
+        <v>37.84</v>
+      </c>
+      <c r="F28" t="n">
+        <v>39.52</v>
+      </c>
+      <c r="G28" t="n">
+        <v>38.64</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1.394</v>
+      </c>
+      <c r="J28" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="K28" t="n">
+        <v>36.09</v>
+      </c>
+      <c r="L28" t="n">
+        <v>4.74</v>
+      </c>
+      <c r="M28" t="n">
+        <v>32777.48</v>
+      </c>
+      <c r="N28" t="n">
+        <v>45574.88</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="P28" t="n">
+        <v>35.55</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>37.82</v>
+      </c>
+      <c r="R28" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>600219</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>南山铝业</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E29" t="n">
+        <v>6.74</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="G29" t="n">
+        <v>6.67</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.455</v>
+      </c>
+      <c r="J29" t="n">
+        <v>25.48</v>
+      </c>
+      <c r="K29" t="n">
+        <v>39.77</v>
+      </c>
+      <c r="L29" t="n">
+        <v>-3.09</v>
+      </c>
+      <c r="M29" t="n">
+        <v>34105.53</v>
+      </c>
+      <c r="N29" t="n">
+        <v>47523.92</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="P29" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="R29" t="n">
+        <v>6.29</v>
+      </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>601939</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>建设银行</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E30" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="F30" t="n">
+        <v>8.74</v>
+      </c>
+      <c r="G30" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-0.081</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-0.091</v>
+      </c>
+      <c r="J30" t="n">
+        <v>60.35</v>
+      </c>
+      <c r="K30" t="n">
+        <v>43.24</v>
+      </c>
+      <c r="L30" t="n">
+        <v>94.56</v>
+      </c>
+      <c r="M30" t="n">
+        <v>9995.82</v>
+      </c>
+      <c r="N30" t="n">
+        <v>11613.78</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="P30" t="n">
+        <v>8.84</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>8.890000000000001</v>
+      </c>
+      <c r="R30" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>600048</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>保利发展</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="D31" t="n">
+        <v>-2.65</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6.95</v>
+      </c>
+      <c r="F31" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="G31" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.167</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.121</v>
+      </c>
+      <c r="J31" t="n">
+        <v>70.97</v>
+      </c>
+      <c r="K31" t="n">
+        <v>69.87</v>
+      </c>
+      <c r="L31" t="n">
+        <v>73.16</v>
+      </c>
+      <c r="M31" t="n">
+        <v>19097.57</v>
+      </c>
+      <c r="N31" t="n">
+        <v>26758.58</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="P31" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>7.15</v>
+      </c>
+      <c r="R31" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>600941</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>中国移动</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>95.11</v>
+      </c>
+      <c r="D32" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="E32" t="n">
+        <v>94.03</v>
+      </c>
+      <c r="F32" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="G32" t="n">
+        <v>96.14</v>
+      </c>
+      <c r="H32" t="n">
+        <v>-1.59</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-1.706</v>
+      </c>
+      <c r="J32" t="n">
+        <v>50.87</v>
+      </c>
+      <c r="K32" t="n">
+        <v>42.76</v>
+      </c>
+      <c r="L32" t="n">
+        <v>67.08</v>
+      </c>
+      <c r="M32" t="n">
+        <v>813.23</v>
+      </c>
+      <c r="N32" t="n">
+        <v>1762.56</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="P32" t="n">
+        <v>95.52</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>95.75</v>
+      </c>
+      <c r="R32" t="n">
+        <v>94.83</v>
+      </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>2352</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>顺丰控股</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>38.86</v>
+      </c>
+      <c r="D33" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="E33" t="n">
+        <v>38.32</v>
+      </c>
+      <c r="F33" t="n">
+        <v>38.15</v>
+      </c>
+      <c r="G33" t="n">
+        <v>38.65</v>
+      </c>
+      <c r="H33" t="n">
+        <v>-0.031</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-0.036</v>
+      </c>
+      <c r="J33" t="n">
+        <v>53.46</v>
+      </c>
+      <c r="K33" t="n">
+        <v>37.78</v>
+      </c>
+      <c r="L33" t="n">
+        <v>84.81</v>
+      </c>
+      <c r="M33" t="n">
+        <v>2897.63</v>
+      </c>
+      <c r="N33" t="n">
+        <v>3540.71</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="P33" t="n">
+        <v>39.01</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>39.42</v>
+      </c>
+      <c r="R33" t="n">
+        <v>38.77</v>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>603803</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>瑞斯康达</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="F34" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="G34" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="H34" t="n">
+        <v>-0.325</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-0.357</v>
+      </c>
+      <c r="J34" t="n">
+        <v>58.75</v>
+      </c>
+      <c r="K34" t="n">
+        <v>45.58</v>
+      </c>
+      <c r="L34" t="n">
+        <v>85.09</v>
+      </c>
+      <c r="M34" t="n">
+        <v>797.6799999999999</v>
+      </c>
+      <c r="N34" t="n">
+        <v>1684.82</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="P34" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>10.23</v>
+      </c>
+      <c r="R34" t="n">
+        <v>9.98</v>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>2624</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>完美世界</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="D35" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="E35" t="n">
+        <v>18.21</v>
+      </c>
+      <c r="F35" t="n">
+        <v>18.15</v>
+      </c>
+      <c r="G35" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="J35" t="n">
+        <v>63.49</v>
+      </c>
+      <c r="K35" t="n">
+        <v>54.26</v>
+      </c>
+      <c r="L35" t="n">
+        <v>81.97</v>
+      </c>
+      <c r="M35" t="n">
+        <v>10719.83</v>
+      </c>
+      <c r="N35" t="n">
+        <v>5608.38</v>
+      </c>
+      <c r="O35" t="n">
+        <v>1.91</v>
+      </c>
+      <c r="P35" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>19.57</v>
+      </c>
+      <c r="R35" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>2558</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>巨人网络</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>42.02</v>
+      </c>
+      <c r="D36" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="E36" t="n">
+        <v>42.04</v>
+      </c>
+      <c r="F36" t="n">
+        <v>43.64</v>
+      </c>
+      <c r="G36" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-0.922</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-0.078</v>
+      </c>
+      <c r="J36" t="n">
+        <v>18.41</v>
+      </c>
+      <c r="K36" t="n">
+        <v>17.87</v>
+      </c>
+      <c r="L36" t="n">
+        <v>19.49</v>
+      </c>
+      <c r="M36" t="n">
+        <v>3769.8</v>
+      </c>
+      <c r="N36" t="n">
+        <v>4414.22</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P36" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>42.87</v>
+      </c>
+      <c r="R36" t="n">
+        <v>40.26</v>
+      </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>601088</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>中国神华</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="D37" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="E37" t="n">
+        <v>41.15</v>
+      </c>
+      <c r="F37" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="G37" t="n">
+        <v>41.14</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.158</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="J37" t="n">
+        <v>63.4</v>
+      </c>
+      <c r="K37" t="n">
+        <v>54.74</v>
+      </c>
+      <c r="L37" t="n">
+        <v>80.70999999999999</v>
+      </c>
+      <c r="M37" t="n">
+        <v>2518.04</v>
+      </c>
+      <c r="N37" t="n">
+        <v>3808.47</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="P37" t="n">
+        <v>41.43</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>42.19</v>
+      </c>
+      <c r="R37" t="n">
+        <v>41.05</v>
+      </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>600963</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>岳阳林纸</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5.92</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="G38" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.368</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.271</v>
+      </c>
+      <c r="J38" t="n">
+        <v>81.29000000000001</v>
+      </c>
+      <c r="K38" t="n">
+        <v>82.45</v>
+      </c>
+      <c r="L38" t="n">
+        <v>78.95999999999999</v>
+      </c>
+      <c r="M38" t="n">
+        <v>10794.4</v>
+      </c>
+      <c r="N38" t="n">
+        <v>7848.04</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="P38" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>6.18</v>
+      </c>
+      <c r="R38" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>601877</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>正泰电器</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>29.87</v>
+      </c>
+      <c r="D39" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>30.25</v>
+      </c>
+      <c r="F39" t="n">
+        <v>30.31</v>
+      </c>
+      <c r="G39" t="n">
+        <v>30.62</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.411</v>
+      </c>
+      <c r="J39" t="n">
+        <v>42.15</v>
+      </c>
+      <c r="K39" t="n">
+        <v>41.38</v>
+      </c>
+      <c r="L39" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="M39" t="n">
+        <v>1811.36</v>
+      </c>
+      <c r="N39" t="n">
+        <v>4322.12</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="P39" t="n">
+        <v>29.63</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>30.39</v>
+      </c>
+      <c r="R39" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
         <is>
           <t>2026-02-06</t>
         </is>

</xml_diff>